<commit_message>
Export-Formen: entfernen nur bei Pflanzen als Stern, Beschriftungen weichen aus
- entfernen: Stern + X nur mit pflanze=true; sonst Hinweis + Pfeil + kleines rotes X
- Eigene Beschriftungen weichen vorhandenen Beschriftungen aus (rechts/unten/links/oben),
  Bau-Formen bleiben unverändert; Überdeckungen durch Körper-Formen werden gemeldet
- Adapter erkennt Pflanzen per Wortliste; Stilprobe und Vergleichsbild neu

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HtoNJ3bRdjfhPeEhztXJF5
</commit_message>
<xml_diff>
--- a/tools/ki-test/ergebnis-skizze/fall1/formen-export.xlsx
+++ b/tools/ki-test/ergebnis-skizze/fall1/formen-export.xlsx
@@ -19560,63 +19560,25 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1538611</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>126716</xdr:rowOff>
+      <xdr:colOff>1754511</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>152116</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>240036</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>114016</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="66" name="Holzpferd" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3367411" y="3441416"/>
-          <a:ext cx="558800" cy="558800"/>
-        </a:xfrm>
-        <a:prstGeom prst="star16">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="70AD47"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1650371</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>47976</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>128276</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>2256</xdr:rowOff>
+      <xdr:colOff>24136</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>88616</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="67" name="Holzpferd_X1" descr="wep-app"/>
+        <xdr:cNvPr id="66" name="Holzpferd_X1" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3479171" y="3553176"/>
-          <a:ext cx="335280" cy="335280"/>
+          <a:off x="3583311" y="3657316"/>
+          <a:ext cx="127000" cy="127000"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -19633,25 +19595,25 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1650371</xdr:colOff>
+      <xdr:colOff>1754511</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>47976</xdr:rowOff>
+      <xdr:rowOff>152116</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>128276</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>2256</xdr:rowOff>
+      <xdr:colOff>24136</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>88616</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="68" name="Holzpferd_X2" descr="wep-app"/>
+        <xdr:cNvPr id="67" name="Holzpferd_X2" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="3479171" y="3553176"/>
-          <a:ext cx="335280" cy="335280"/>
+          <a:off x="3583311" y="3657316"/>
+          <a:ext cx="127000" cy="127000"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -19680,7 +19642,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="69" name="Hochbeete_Text" descr="wep-app"/>
+        <xdr:cNvPr id="68" name="Hochbeete_Text" descr="wep-app"/>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -19719,23 +19681,23 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>1169994</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>152116</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>608654</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>164816</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="70" name="Holzpferd_Hinweis" descr="wep-app"/>
+        <xdr:cNvPr id="69" name="Holzpferd_Hinweis" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2998794" y="3085816"/>
+          <a:off x="2998794" y="3276316"/>
           <a:ext cx="1296035" cy="203200"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -19773,23 +19735,23 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>1818011</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>164816</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>1818011</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>126716</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="71" name="Holzpferd_Pfeil" descr="wep-app"/>
+        <xdr:cNvPr id="70" name="Holzpferd_Pfeil" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3646811" y="3289016"/>
+          <a:off x="3646811" y="3479516"/>
           <a:ext cx="0" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">

</xml_diff>

<commit_message>
Export-Formen: Körper-Formen weichen Bau-Labels und Bau-Formen aus
- Beete/Hochbeete/Kompost/Gegenstände, die ein Bau-Label oder eine Bau-Form überdecken, werden
  als Gruppe minimal versetzt (weg vom Hindernis, <= 1 Elementhöhe), sonst bis 20 % verkleinert
- Bäume/Sträucher/Hecken nie bewegt, nur gemeldet; umschließende Bau-Formen zählen nicht
- Ergebnis meldet versetzt/verkleinert/ueberdeckt; Vergleichsbild neu
- ausrichtung.test an soll.json nach Nachtrag angepasst (Pavillon LVP = LVP)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HtoNJ3bRdjfhPeEhztXJF5
</commit_message>
<xml_diff>
--- a/tools/ki-test/ergebnis-skizze/fall1/formen-export.xlsx
+++ b/tools/ki-test/ergebnis-skizze/fall1/formen-export.xlsx
@@ -19407,16 +19407,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1186031</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>101315</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>351860</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>183692</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>148008</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>148435</xdr:rowOff>
+      <xdr:colOff>530874</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>107088</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -19425,8 +19425,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1795631" y="6654515"/>
-          <a:ext cx="181177" cy="618620"/>
+          <a:off x="2180660" y="6546392"/>
+          <a:ext cx="179014" cy="494896"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -19446,15 +19446,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>278623</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>101315</xdr:rowOff>
+      <xdr:colOff>659931</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>183692</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>426092</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>136538</xdr:rowOff>
+      <xdr:colOff>805641</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>97570</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -19463,8 +19463,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2107423" y="6654515"/>
-          <a:ext cx="147469" cy="606723"/>
+          <a:off x="2488731" y="6546392"/>
+          <a:ext cx="145710" cy="485378"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -19484,15 +19484,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>682283</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>101315</xdr:rowOff>
+      <xdr:colOff>992981</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>183692</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>879782</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>65159</xdr:rowOff>
+      <xdr:colOff>1126201</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>40467</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -19501,8 +19501,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2511083" y="6654515"/>
-          <a:ext cx="197499" cy="535344"/>
+          <a:off x="2821781" y="6546392"/>
+          <a:ext cx="133220" cy="428275"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -19522,15 +19522,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>978532</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>41832</xdr:rowOff>
+      <xdr:colOff>1192811</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>136106</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1225406</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>65159</xdr:rowOff>
+      <xdr:colOff>1359336</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>40468</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -19539,8 +19539,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2807332" y="6595032"/>
-          <a:ext cx="246874" cy="594827"/>
+          <a:off x="3021611" y="6498806"/>
+          <a:ext cx="166525" cy="475862"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
@@ -19560,13 +19560,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1754511</xdr:colOff>
+      <xdr:colOff>1832745</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>152116</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>24136</xdr:colOff>
+      <xdr:colOff>102370</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>88616</xdr:rowOff>
     </xdr:to>
@@ -19577,7 +19577,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3583311" y="3657316"/>
+          <a:off x="3661545" y="3657316"/>
           <a:ext cx="127000" cy="127000"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -19595,13 +19595,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1754511</xdr:colOff>
+      <xdr:colOff>1832745</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>152116</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>24136</xdr:colOff>
+      <xdr:colOff>102370</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>88616</xdr:rowOff>
     </xdr:to>
@@ -19612,7 +19612,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="3583311" y="3657316"/>
+          <a:off x="3661545" y="3657316"/>
           <a:ext cx="127000" cy="127000"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -19630,15 +19630,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1263506</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>95133</xdr:rowOff>
+      <xdr:colOff>1523370</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>121597</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>79231</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>95133</xdr:rowOff>
+      <xdr:colOff>339095</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>121597</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -19647,7 +19647,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3092306" y="6838833"/>
+          <a:off x="3352170" y="6674797"/>
           <a:ext cx="673100" cy="190500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -19680,13 +19680,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1169994</xdr:colOff>
+      <xdr:colOff>1248228</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>152116</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>608654</xdr:colOff>
+      <xdr:colOff>686888</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>164816</xdr:rowOff>
     </xdr:to>
@@ -19697,7 +19697,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2998794" y="3276316"/>
+          <a:off x="3077028" y="3276316"/>
           <a:ext cx="1296035" cy="203200"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
@@ -19733,14 +19733,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1818011</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>38870</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>164816</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1818011</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>38870</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>126716</xdr:rowOff>
     </xdr:to>
@@ -19751,7 +19751,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3646811" y="3479516"/>
+          <a:off x="3725045" y="3479516"/>
           <a:ext cx="0" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">

</xml_diff>